<commit_message>
Daily slate 2026-06-22 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-06-20.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-06-20.xlsx
@@ -471,16 +471,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="E2" t="n">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="F2" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="G2" t="n">
-        <v>57.4</v>
+        <v>57.5</v>
       </c>
     </row>
     <row r="3">
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>406</v>
+        <v>414</v>
       </c>
       <c r="E4" t="n">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="F4" t="n">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="G4" t="n">
-        <v>39.2</v>
+        <v>39.4</v>
       </c>
     </row>
     <row r="5">
@@ -616,16 +616,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="E7" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="F7" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="G7" t="n">
-        <v>42.1</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8">
@@ -674,16 +674,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E9" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F9" t="n">
         <v>20</v>
       </c>
       <c r="G9" t="n">
-        <v>52.4</v>
+        <v>53.5</v>
       </c>
     </row>
     <row r="10">
@@ -703,16 +703,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="E10" t="n">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F10" t="n">
         <v>157</v>
       </c>
       <c r="G10" t="n">
-        <v>47.7</v>
+        <v>48</v>
       </c>
     </row>
     <row r="11">
@@ -732,16 +732,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>977</v>
+        <v>1042</v>
       </c>
       <c r="E11" t="n">
-        <v>576</v>
+        <v>611</v>
       </c>
       <c r="F11" t="n">
-        <v>401</v>
+        <v>431</v>
       </c>
       <c r="G11" t="n">
-        <v>59</v>
+        <v>58.6</v>
       </c>
     </row>
     <row r="12">
@@ -761,13 +761,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="E12" t="n">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="F12" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="G12" t="n">
         <v>66.7</v>
@@ -819,16 +819,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>316</v>
+        <v>324</v>
       </c>
       <c r="E14" t="n">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="F14" t="n">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="G14" t="n">
-        <v>29.1</v>
+        <v>29.3</v>
       </c>
     </row>
     <row r="15">
@@ -848,16 +848,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>385</v>
+        <v>396</v>
       </c>
       <c r="E15" t="n">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F15" t="n">
-        <v>303</v>
+        <v>312</v>
       </c>
       <c r="G15" t="n">
-        <v>21.3</v>
+        <v>21.2</v>
       </c>
     </row>
     <row r="16">
@@ -877,16 +877,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="E16" t="n">
         <v>38</v>
       </c>
       <c r="F16" t="n">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="G16" t="n">
-        <v>21</v>
+        <v>20.3</v>
       </c>
     </row>
     <row r="17">
@@ -906,16 +906,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>4810</v>
+        <v>5091</v>
       </c>
       <c r="E17" t="n">
-        <v>897</v>
+        <v>939</v>
       </c>
       <c r="F17" t="n">
-        <v>3913</v>
+        <v>4152</v>
       </c>
       <c r="G17" t="n">
-        <v>18.6</v>
+        <v>18.4</v>
       </c>
     </row>
   </sheetData>
@@ -1507,22 +1507,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>47.7</v>
+        <v>48</v>
       </c>
       <c r="C7" t="n">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="D7" t="n">
-        <v>59</v>
+        <v>58.6</v>
       </c>
       <c r="E7" t="n">
-        <v>977</v>
+        <v>1042</v>
       </c>
       <c r="F7" t="n">
         <v>66.7</v>
       </c>
       <c r="G7" t="n">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="H7" t="n">
         <v>56.2</v>
@@ -1531,40 +1531,40 @@
         <v>64</v>
       </c>
       <c r="J7" t="n">
-        <v>29.1</v>
+        <v>29.3</v>
       </c>
       <c r="K7" t="n">
-        <v>316</v>
+        <v>324</v>
       </c>
       <c r="L7" t="n">
-        <v>21.3</v>
+        <v>21.2</v>
       </c>
       <c r="M7" t="n">
-        <v>385</v>
+        <v>396</v>
       </c>
       <c r="N7" t="n">
-        <v>21</v>
+        <v>20.3</v>
       </c>
       <c r="O7" t="n">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="P7" t="n">
-        <v>18.6</v>
+        <v>18.4</v>
       </c>
       <c r="Q7" t="n">
-        <v>4810</v>
+        <v>5091</v>
       </c>
       <c r="R7" t="n">
-        <v>57.4</v>
+        <v>57.5</v>
       </c>
       <c r="S7" t="n">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="T7" t="n">
-        <v>39.2</v>
+        <v>39.4</v>
       </c>
       <c r="U7" t="n">
-        <v>406</v>
+        <v>414</v>
       </c>
       <c r="V7" t="n">
         <v>50</v>
@@ -1591,16 +1591,16 @@
         <v>43</v>
       </c>
       <c r="AD7" t="n">
-        <v>42.1</v>
+        <v>43</v>
       </c>
       <c r="AE7" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="AF7" t="n">
-        <v>52.4</v>
+        <v>53.5</v>
       </c>
       <c r="AG7" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>